<commit_message>
Make job matching candidate-driven
</commit_message>
<xml_diff>
--- a/examples/demo_ranking.xlsx
+++ b/examples/demo_ranking.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'建议投递排名'!$A$1:$Q$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'建议投递排名'!$A$1:$V$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q6"/>
+  <dimension ref="A1:V7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -457,16 +457,21 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="8" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="38" customWidth="1" min="15" max="15"/>
-    <col width="38" customWidth="1" min="16" max="16"/>
-    <col width="26" customWidth="1" min="17" max="17"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
+    <col width="8" customWidth="1" min="18" max="18"/>
+    <col width="14" customWidth="1" min="19" max="19"/>
+    <col width="38" customWidth="1" min="20" max="20"/>
+    <col width="38" customWidth="1" min="21" max="21"/>
+    <col width="26" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -502,55 +507,80 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>届次</t>
+          <t>届次(岗位)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>学历</t>
+          <t>届次匹配</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>学历(岗位)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>学历匹配</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>专业相关</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>岗位方向证据</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>核心缺口</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
           <t>截止</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>命中关键词</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>弱证据</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>缺口</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>JD已核实</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>建议</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>投递链接</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>公告链接</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>定制简历</t>
         </is>
@@ -561,21 +591,21 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>某商业银行</t>
+          <t>某咨询公司</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>管理培训生（金融市场方向、公司金融方向、风险合规方向）</t>
+          <t>金融咨询顾问（风险管理、财务转型）</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>上海, 深圳</t>
+          <t>北京, 深圳</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -590,67 +620,88 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>本科、硕士</t>
+          <t>是（2026届）</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>2026-12-31</t>
+          <t>本科、硕士、博士</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>财务分析、分析、风险、合规、数据</t>
+          <t>是（本科）</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>数据分析</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr"/>
-      <c r="M2" s="2" t="inlineStr">
+          <t>相关（仅提示）</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>有可迁移证据：finance、business</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>尽快投递</t>
+        </is>
+      </c>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>财务、风险、金融</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>咨询、顾问</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="N2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>优先投</t>
         </is>
       </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>https://example.com/a</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
-        <is>
-          <t>https://example.com/a-notice</t>
-        </is>
-      </c>
-      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/d</t>
+        </is>
+      </c>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/d-notice</t>
+        </is>
+      </c>
+      <c r="V2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>某证券公司</t>
+          <t>某制造企业</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>固定收益部-债券承做助理、信用研究助理</t>
+          <t>财务管理岗（预算与经营分析）</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>北京, 上海</t>
+          <t>苏州</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -660,147 +711,185 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
+          <t>2026届</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>是（2026届）</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>是（本科）</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>相关（仅提示）</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>有可迁移证据：finance</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>财务、预算、分析</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>经营分析、成本分析</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr">
+        <is>
+          <t>优先投</t>
+        </is>
+      </c>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/e</t>
+        </is>
+      </c>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/e-notice</t>
+        </is>
+      </c>
+      <c r="V3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>某商业银行</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>管理培训生（金融市场方向、公司金融方向、风险合规方向）</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>上海, 深圳</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
           <t>2027届, 2026届</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>是（2026届）</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>本科、硕士</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>分析、研究、定价、债券、久期</t>
-        </is>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>信用分析</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr"/>
-      <c r="M3" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>是（本科）</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>相关（仅提示）</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>有可迁移证据：finance、compliance、business</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr">
+        <is>
+          <t>2026-12-31</t>
+        </is>
+      </c>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>风险、合规、金融</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr">
+      <c r="S4" s="2" t="inlineStr">
         <is>
           <t>优先投</t>
         </is>
       </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>https://example.com/b</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
-        <is>
-          <t>https://example.com/b-notice</t>
-        </is>
-      </c>
-      <c r="Q3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>67</v>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>某制造企业</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>财务管理岗（预算与经营分析）</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>苏州</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>2026届</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>本科</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>2026-11-20</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>预算、差异分析、分析</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>经营分析、成本分析</t>
-        </is>
-      </c>
-      <c r="L4" s="3" t="inlineStr"/>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
-      </c>
-      <c r="N4" s="3" t="inlineStr">
-        <is>
-          <t>可投</t>
-        </is>
-      </c>
-      <c r="O4" s="3" t="inlineStr">
-        <is>
-          <t>https://example.com/e</t>
-        </is>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>https://example.com/e-notice</t>
-        </is>
-      </c>
-      <c r="Q4" s="3" t="inlineStr"/>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/a</t>
+        </is>
+      </c>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>https://example.com/a-notice</t>
+        </is>
+      </c>
+      <c r="V4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>某咨询公司</t>
+          <t>某证券公司</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>金融咨询顾问（风险管理、财务转型）</t>
+          <t>固定收益部-债券承做助理、信用研究助理</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>北京, 深圳</t>
+          <t>北京, 上海</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -815,57 +904,74 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>本科、硕士、博士</t>
+          <t>是（2026届）</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>尽快投递</t>
+          <t>本科、硕士</t>
         </is>
       </c>
       <c r="J5" s="3" t="inlineStr">
         <is>
-          <t>财务分析、分析、风险、数据</t>
+          <t>是（本科）</t>
         </is>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>数据分析</t>
+          <t>相关（仅提示）</t>
         </is>
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>咨询、顾问</t>
-        </is>
-      </c>
-      <c r="M5" s="3" t="inlineStr">
+          <t>有可迁移证据：finance</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="inlineStr"/>
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-30</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="inlineStr">
+        <is>
+          <t>债券、金融</t>
+        </is>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>研究</t>
+        </is>
+      </c>
+      <c r="Q5" s="3" t="inlineStr"/>
+      <c r="R5" s="3" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="N5" s="3" t="inlineStr">
+      <c r="S5" s="3" t="inlineStr">
         <is>
           <t>可投</t>
         </is>
       </c>
-      <c r="O5" s="3" t="inlineStr">
-        <is>
-          <t>https://example.com/d</t>
-        </is>
-      </c>
-      <c r="P5" s="3" t="inlineStr">
-        <is>
-          <t>https://example.com/d-notice</t>
-        </is>
-      </c>
-      <c r="Q5" s="3" t="inlineStr"/>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>https://example.com/b</t>
+        </is>
+      </c>
+      <c r="U5" s="3" t="inlineStr">
+        <is>
+          <t>https://example.com/b-notice</t>
+        </is>
+      </c>
+      <c r="V5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>52</v>
+        <v>33</v>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
@@ -894,49 +1000,170 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
+          <t>是（2026届）</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
           <t>本科、硕士</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>是（本科）</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>相关（仅提示）</t>
+        </is>
+      </c>
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>有可迁移证据：finance</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="inlineStr"/>
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>2026-12-15</t>
         </is>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>勾稽</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>底稿、审计</t>
-        </is>
-      </c>
-      <c r="L6" s="3" t="inlineStr"/>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="O6" s="3" t="inlineStr">
+        <is>
+          <t>金融</t>
+        </is>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>审计</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr"/>
+      <c r="R6" s="3" t="inlineStr">
         <is>
           <t>否</t>
         </is>
       </c>
-      <c r="N6" s="3" t="inlineStr">
-        <is>
-          <t>可投</t>
-        </is>
-      </c>
-      <c r="O6" s="3" t="inlineStr">
+      <c r="S6" s="3" t="inlineStr">
+        <is>
+          <t>备选</t>
+        </is>
+      </c>
+      <c r="T6" s="3" t="inlineStr">
         <is>
           <t>https://example.com/c</t>
         </is>
       </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="U6" s="3" t="inlineStr">
         <is>
           <t>https://example.com/c-notice</t>
         </is>
       </c>
-      <c r="Q6" s="3" t="inlineStr"/>
+      <c r="V6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>某科技公司</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>AI 算法工程师</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>深圳</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>2026届</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>是（2026届）</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>本科、硕士</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>是（本科）</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>不匹配（仅提示）</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr">
+        <is>
+          <t>有可迁移证据：technology</t>
+        </is>
+      </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>算法</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="inlineStr">
+        <is>
+          <t>2026-11-20</t>
+        </is>
+      </c>
+      <c r="O7" s="3" t="inlineStr">
+        <is>
+          <t>AI</t>
+        </is>
+      </c>
+      <c r="P7" s="3" t="inlineStr"/>
+      <c r="Q7" s="3" t="inlineStr">
+        <is>
+          <t>算法</t>
+        </is>
+      </c>
+      <c r="R7" s="3" t="inlineStr">
+        <is>
+          <t>否</t>
+        </is>
+      </c>
+      <c r="S7" s="3" t="inlineStr">
+        <is>
+          <t>备选</t>
+        </is>
+      </c>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>https://example.com/f</t>
+        </is>
+      </c>
+      <c r="U7" s="3" t="inlineStr">
+        <is>
+          <t>https://example.com/f-notice</t>
+        </is>
+      </c>
+      <c r="V7" s="3" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q6"/>
+  <autoFilter ref="A1:V7"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -947,7 +1174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -974,33 +1201,6 @@
       <c r="E1" s="4" t="inlineStr">
         <is>
           <t>排除原因</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>某科技公司</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>AI 算法工程师</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>深圳</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>2026-11-20</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>非金融/财务目标域</t>
         </is>
       </c>
     </row>
@@ -1015,10 +1215,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -1040,83 +1240,195 @@
           <t>简历来源</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>data/profile.json</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>岗位总数</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>6</v>
+          <t>毕业时间</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>进入排名</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>5</v>
+          <t>届次（推算）</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026 届</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>已排除</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
+          <t>学历</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>本科</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>硬过滤</t>
+          <t>专业</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>学历含本科；届次含 2026（若有）；截止未过（或尽快/长期）</t>
+          <t>金融</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>打分</t>
+          <t>届次规则</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>岗位文本里的关键词 × 简历证据：强命中 1 分、弱证据 0.5 分，折算百分制</t>
+          <t>毕业月份 ≥ 9 月归入下一年届（2025-12 / 2026-01 → 2026 届）</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>深度核实</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>对前 0 个有链接的岗位抓取 JD 后重算</t>
-        </is>
+          <t>岗位总数</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>进入排名</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>已排除</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>硬过滤</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>身份条件：本人届次、本人学历；过期或无可用关键词的岗位也会排除</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>专业</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>只做提示，不设门槛，也不改匹配分</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>技术岗</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>不排除；开发、算法、数据等岗位与金融岗位使用同一套证据打分</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>岗位方向</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>简历完全无对应方向证据时封顶 35，仍保留供人工查看</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>词权重</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>关键词基础权重 × 该能力在简历经历/项目中的证据强度</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>泛词处理</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>分析、数据、团队、沟通等泛词降权且限制动态放大</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>覆盖折扣</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>岗位可用关键词总权重不足 10 时按比例打折</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>注意</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>岗位字段常含多个职位，投前点开链接核对；分数用于排序，不替代人工判断</t>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>岗位字段常含多个职位，投前点开链接核对</t>
         </is>
       </c>
     </row>

</xml_diff>